<commit_message>
Add authentication and authorization to estore-backend
Implemented JWT-based authentication and authorization, including login and signup endpoints, JWT utility and filter, and security configuration. Added user, role, and permission models with repositories and service logic. Updated exception handling, logging configuration, and application properties for JWT settings. Enhanced entity classes with Lombok annotations and improved equals/hashCode implementations.
</commit_message>
<xml_diff>
--- a/Document/Techincal/FitLux_API_Endpoints.xlsx
+++ b/Document/Techincal/FitLux_API_Endpoints.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="23040" windowHeight="8555"/>
   </bookViews>
   <sheets>
     <sheet name="API_Endpoints Finished" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="19">
   <si>
     <t>Module</t>
   </si>
@@ -47,334 +47,43 @@
     <t>File Path</t>
   </si>
   <si>
+    <t>Authenticated</t>
+  </si>
+  <si>
     <t>Users</t>
   </si>
   <si>
+    <t xml:space="preserve">GET </t>
+  </si>
+  <si>
+    <t>/api/public/products</t>
+  </si>
+  <si>
+    <t>/api/public/products/{id}</t>
+  </si>
+  <si>
+    <t>/api/public/categories</t>
+  </si>
+  <si>
+    <t>/api/public/brands</t>
+  </si>
+  <si>
     <t>POST</t>
   </si>
   <si>
-    <t>/user/register</t>
-  </si>
-  <si>
-    <t>body userDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Register user</t>
-  </si>
-  <si>
-    <t>usersController.java</t>
-  </si>
-  <si>
-    <t>/user/login</t>
-  </si>
-  <si>
-    <t>body EncryptedDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Login user</t>
-  </si>
-  <si>
-    <t>/user/signout</t>
-  </si>
-  <si>
-    <t>header Request-id</t>
-  </si>
-  <si>
-    <t>Logout user</t>
+    <t xml:space="preserve"> /api/auth/login</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> /api/auth/signup</t>
+  </si>
+  <si>
+    <t>GET</t>
   </si>
   <si>
     <t>DELETE</t>
   </si>
   <si>
-    <t>/user/delete</t>
-  </si>
-  <si>
-    <t>Delete user</t>
-  </si>
-  <si>
-    <t>GET</t>
-  </si>
-  <si>
-    <t>/user/checkUser</t>
-  </si>
-  <si>
-    <t>Check user session</t>
-  </si>
-  <si>
-    <t>Orders</t>
-  </si>
-  <si>
-    <t>/order/placed</t>
-  </si>
-  <si>
-    <t>body OrderDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Place order</t>
-  </si>
-  <si>
-    <t>orderController.java</t>
-  </si>
-  <si>
-    <t>/order/placed/coupon</t>
-  </si>
-  <si>
-    <t>Place order with coupon</t>
-  </si>
-  <si>
-    <t>/order/orders</t>
-  </si>
-  <si>
-    <t>header Request-id, query page, size</t>
-  </si>
-  <si>
-    <t>List orders</t>
-  </si>
-  <si>
-    <t>/order/history</t>
-  </si>
-  <si>
-    <t>Order history custom date</t>
-  </si>
-  <si>
-    <t>/order/ProductList</t>
-  </si>
-  <si>
-    <t>List products in order</t>
-  </si>
-  <si>
-    <t>/order/Product</t>
-  </si>
-  <si>
-    <t>Return product</t>
-  </si>
-  <si>
-    <t>Products</t>
-  </si>
-  <si>
-    <t>/products/upload</t>
-  </si>
-  <si>
-    <t>body List&lt;productRequestDto&gt;, header Request-id</t>
-  </si>
-  <si>
-    <t>Add products</t>
-  </si>
-  <si>
-    <t>productController.java</t>
-  </si>
-  <si>
-    <t>/products/UploadMultiple</t>
-  </si>
-  <si>
-    <t>file MultipartFile, header Request-id</t>
-  </si>
-  <si>
-    <t>Bulk upload products</t>
-  </si>
-  <si>
-    <t>/products/products</t>
-  </si>
-  <si>
-    <t>List products</t>
-  </si>
-  <si>
-    <t>/products/{p_id}</t>
-  </si>
-  <si>
-    <t>header Request-id, path p_id</t>
-  </si>
-  <si>
-    <t>Product details</t>
-  </si>
-  <si>
-    <t>/products/delete</t>
-  </si>
-  <si>
-    <t>body productRequestDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Delete product</t>
-  </si>
-  <si>
-    <t>/products/category</t>
-  </si>
-  <si>
-    <t>Fetch by category</t>
-  </si>
-  <si>
     <t>PATCH</t>
-  </si>
-  <si>
-    <t>/products/updateQuantity</t>
-  </si>
-  <si>
-    <t>Update quantity</t>
-  </si>
-  <si>
-    <t>Cart</t>
-  </si>
-  <si>
-    <t>/cart/productAdd</t>
-  </si>
-  <si>
-    <t>Add to cart</t>
-  </si>
-  <si>
-    <t>cartController.java</t>
-  </si>
-  <si>
-    <t>/cart/productDelete/{PId}</t>
-  </si>
-  <si>
-    <t>header Request-id, path PId</t>
-  </si>
-  <si>
-    <t>Remove product</t>
-  </si>
-  <si>
-    <t>/cart/products</t>
-  </si>
-  <si>
-    <t>List cart products</t>
-  </si>
-  <si>
-    <t>/cart/quantity</t>
-  </si>
-  <si>
-    <t>Update cart quantity</t>
-  </si>
-  <si>
-    <t>/cart/bill</t>
-  </si>
-  <si>
-    <t>Generate cart bill</t>
-  </si>
-  <si>
-    <t>Dashboard</t>
-  </si>
-  <si>
-    <t>/dashboard/</t>
-  </si>
-  <si>
-    <t>body dashboardRequestDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Fetch dashboard metrics</t>
-  </si>
-  <si>
-    <t>dashboardController.java</t>
-  </si>
-  <si>
-    <t>Invoices</t>
-  </si>
-  <si>
-    <t>/invoice/generate</t>
-  </si>
-  <si>
-    <t>body InvoiceRequestDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Generate invoice PDF</t>
-  </si>
-  <si>
-    <t>InvoiceController.java</t>
-  </si>
-  <si>
-    <t>/invoice/invoices/{orderId}</t>
-  </si>
-  <si>
-    <t>path orderId</t>
-  </si>
-  <si>
-    <t>Download invoice PDF</t>
-  </si>
-  <si>
-    <t>Sellers</t>
-  </si>
-  <si>
-    <t>/seller/register</t>
-  </si>
-  <si>
-    <t>body sellerRequestDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Register seller</t>
-  </si>
-  <si>
-    <t>sellerController.java</t>
-  </si>
-  <si>
-    <t>Roles</t>
-  </si>
-  <si>
-    <t>/roles/register</t>
-  </si>
-  <si>
-    <t>body rolesDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Add role</t>
-  </si>
-  <si>
-    <t>rolesController.java</t>
-  </si>
-  <si>
-    <t>/roles/delete</t>
-  </si>
-  <si>
-    <t>Delete role</t>
-  </si>
-  <si>
-    <t>Coupons</t>
-  </si>
-  <si>
-    <t>/coupon/create</t>
-  </si>
-  <si>
-    <t>body couponRequestDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Create coupon</t>
-  </si>
-  <si>
-    <t>couponController.java</t>
-  </si>
-  <si>
-    <t>/coupon/fetchList</t>
-  </si>
-  <si>
-    <t>Get active coupons</t>
-  </si>
-  <si>
-    <t>/coupon/ApplyCoupon</t>
-  </si>
-  <si>
-    <t>Apply coupon</t>
-  </si>
-  <si>
-    <t>/coupon/removeCoupon</t>
-  </si>
-  <si>
-    <t>body PagingDto, header Request-id</t>
-  </si>
-  <si>
-    <t>Remove coupon</t>
-  </si>
-  <si>
-    <t>Encryption</t>
-  </si>
-  <si>
-    <t>/encrypt</t>
-  </si>
-  <si>
-    <t>body Map&lt;String,Object&gt;</t>
-  </si>
-  <si>
-    <t>Encrypt payload</t>
-  </si>
-  <si>
-    <t>encryptController.java</t>
   </si>
 </sst>
 </file>
@@ -1054,7 +763,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1067,6 +776,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1492,18 +1207,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="5"/>
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
     <col min="4" max="4" width="52" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="6" max="7" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1522,643 +1237,401 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="5"/>
       <c r="B3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="5"/>
       <c r="B4" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="5"/>
       <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="6"/>
+        <v>12</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="5"/>
       <c r="B6" s="3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="5"/>
       <c r="B7" s="3" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>15</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="5"/>
       <c r="B8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>13</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="5"/>
       <c r="B9" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>16</v>
+      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="5"/>
       <c r="B10" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>16</v>
+      </c>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="5"/>
       <c r="B11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>13</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" s="5"/>
       <c r="B12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="2" t="s">
-        <v>40</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="6"/>
       <c r="B13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="5"/>
+        <v>13</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="7"/>
       <c r="B14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="5"/>
+        <v>13</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="7"/>
       <c r="B15" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="5"/>
+        <v>16</v>
+      </c>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="7"/>
       <c r="B16" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="5"/>
+        <v>16</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="7"/>
       <c r="B17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="7"/>
+      <c r="B18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="8"/>
+      <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="5"/>
-      <c r="B18" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="6"/>
-      <c r="B19" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="2" t="s">
-        <v>61</v>
-      </c>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="6"/>
       <c r="B20" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="5"/>
+        <v>13</v>
+      </c>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="7"/>
       <c r="B21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="7"/>
+      <c r="B22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="7"/>
+      <c r="B23" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="5"/>
-      <c r="B22" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" s="5"/>
-      <c r="B23" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="6"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="8"/>
       <c r="B24" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="D24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="6"/>
       <c r="B26" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="6"/>
+        <v>13</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="8"/>
       <c r="B27" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="3" t="s">
-        <v>87</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="3"/>
       <c r="B28" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="2" t="s">
-        <v>92</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="6"/>
       <c r="B29" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" s="6"/>
+        <v>13</v>
+      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="8"/>
       <c r="B30" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F30" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="2" t="s">
-        <v>99</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="6"/>
       <c r="B31" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="F31" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="5"/>
+        <v>13</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="7"/>
       <c r="B32" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D32" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E32" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="5"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="7"/>
       <c r="B33" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="6"/>
+        <v>13</v>
+      </c>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="8"/>
       <c r="B34" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="3" t="s">
-        <v>111</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="3"/>
       <c r="B35" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>115</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A7:A12"/>
+  <mergeCells count="6">
+    <mergeCell ref="A2:A12"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="A20:A24"/>
     <mergeCell ref="A26:A27"/>
@@ -2166,18 +1639,23 @@
     <mergeCell ref="A31:A34"/>
   </mergeCells>
   <conditionalFormatting sqref="B$1:B$1048576">
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
       <formula>"POST"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"DELETE"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"GET"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G$1:G$1048576">
+    <cfRule type="cellIs" priority="1" operator="equal">
+      <formula>"YES,NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B35">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B7 B8:B35">
       <formula1>"GET,PUT,POST,PATCH,DELETE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>